<commit_message>
feat: Unified optimization architecture v2.0.0
- Consolidated 5 scripts into 2 unified scripts with multiple modes
- Main script: optimize_coft.sh (diagnostic, quick, optimize, help modes)
- Colab script: optimize_coft_colab.sh (Colab-optimized version)
- Removed broken/duplicate scripts and cleaned up file clutter
- Enhanced UX with color output and mode-based execution
- Updated documentation (README, CHANGELOG) for v2.0.0
- Clean architecture ready for production use
</commit_message>
<xml_diff>
--- a/experiments_logs/HAR_experiments/test1/ft_1p_seed_0/test1_ft_1p_seed_0_classification_report.xlsx
+++ b/experiments_logs/HAR_experiments/test1/ft_1p_seed_0/test1_ft_1p_seed_0_classification_report.xlsx
@@ -487,34 +487,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60.18237082066869</v>
+        <v>62.47689463955638</v>
       </c>
       <c r="C2" t="n">
         <v>100</v>
       </c>
       <c r="D2" t="n">
-        <v>30.85376162299239</v>
+        <v>28.49462365591398</v>
       </c>
       <c r="E2" t="n">
-        <v>78.125</v>
+        <v>82.60869565217391</v>
       </c>
       <c r="F2" t="n">
-        <v>78.78151260504201</v>
+        <v>81.80039138943248</v>
       </c>
       <c r="G2" t="n">
-        <v>96.38989169675091</v>
+        <v>96.03603603603604</v>
       </c>
       <c r="H2" t="n">
-        <v>58.77163216830675</v>
+        <v>57.48218527315915</v>
       </c>
       <c r="I2" t="n">
-        <v>74.05542279090901</v>
+        <v>75.23610689551879</v>
       </c>
       <c r="J2" t="n">
-        <v>75.31101030055855</v>
+        <v>76.58850044535143</v>
       </c>
       <c r="K2" t="n">
-        <v>50.77377290334111</v>
+        <v>49.28726501046229</v>
       </c>
     </row>
     <row r="3">
@@ -524,34 +524,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>79.83870967741935</v>
+        <v>68.14516129032258</v>
       </c>
       <c r="C3" t="n">
-        <v>2.547770700636943</v>
+        <v>3.184713375796179</v>
       </c>
       <c r="D3" t="n">
-        <v>86.90476190476191</v>
+        <v>88.33333333333333</v>
       </c>
       <c r="E3" t="n">
-        <v>10.18329938900204</v>
+        <v>3.869653767820774</v>
       </c>
       <c r="F3" t="n">
-        <v>70.48872180451127</v>
+        <v>78.57142857142857</v>
       </c>
       <c r="G3" t="n">
-        <v>99.44134078212289</v>
+        <v>99.25512104283054</v>
       </c>
       <c r="H3" t="n">
-        <v>58.77163216830675</v>
+        <v>57.48218527315915</v>
       </c>
       <c r="I3" t="n">
-        <v>58.23410070974241</v>
+        <v>56.89323523025532</v>
       </c>
       <c r="J3" t="n">
-        <v>58.77163216830675</v>
+        <v>57.48218527315915</v>
       </c>
       <c r="K3" t="n">
-        <v>50.77377290334111</v>
+        <v>49.28726501046229</v>
       </c>
     </row>
     <row r="4">
@@ -561,34 +561,34 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>68.63084922010398</v>
+        <v>65.18804243008678</v>
       </c>
       <c r="C4" t="n">
-        <v>4.968944099378882</v>
+        <v>6.17283950617284</v>
       </c>
       <c r="D4" t="n">
-        <v>45.53961322520274</v>
+        <v>43.08943089430895</v>
       </c>
       <c r="E4" t="n">
-        <v>18.01801801801802</v>
+        <v>7.392996108949417</v>
       </c>
       <c r="F4" t="n">
-        <v>74.40476190476191</v>
+        <v>80.15340364333653</v>
       </c>
       <c r="G4" t="n">
-        <v>97.89184234647112</v>
+        <v>97.61904761904762</v>
       </c>
       <c r="H4" t="n">
-        <v>58.77163216830675</v>
+        <v>57.48218527315915</v>
       </c>
       <c r="I4" t="n">
-        <v>51.57567146898945</v>
+        <v>49.93596003365035</v>
       </c>
       <c r="J4" t="n">
-        <v>53.10689207967404</v>
+        <v>51.58847567951068</v>
       </c>
       <c r="K4" t="n">
-        <v>50.77377290334111</v>
+        <v>49.28726501046229</v>
       </c>
     </row>
     <row r="5">
@@ -616,7 +616,7 @@
         <v>53700</v>
       </c>
       <c r="H5" t="n">
-        <v>58.77163216830675</v>
+        <v>57.48218527315915</v>
       </c>
       <c r="I5" t="n">
         <v>294700</v>
@@ -625,7 +625,7 @@
         <v>294700</v>
       </c>
       <c r="K5" t="n">
-        <v>50.77377290334111</v>
+        <v>49.28726501046229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>